<commit_message>
Se actualiza Sitios para Seguimiento
</commit_message>
<xml_diff>
--- a/data/Sitios3G.xlsx
+++ b/data/Sitios3G.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonat\project\dashboard\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonat\Documents\project\ubuntu\dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{327CE0F4-8A9B-482E-89DA-2D7BFB60F586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A24DA865-3495-4242-8970-1FD63AAD3501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{4309663C-230E-4C6A-A396-815C205117AE}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4309663C-230E-4C6A-A396-815C205117AE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sitios" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2427" uniqueCount="2034">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2429" uniqueCount="2033">
   <si>
     <t>CHI_RIO_SC_MIES_U</t>
   </si>
@@ -6029,9 +6029,6 @@
   </si>
   <si>
     <t>Sitio</t>
-  </si>
-  <si>
-    <t>SMALL_UIO_REPUBLICAL21</t>
   </si>
   <si>
     <t>ORO_MCH_ARAUJO_UL</t>
@@ -7170,7 +7167,7 @@
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>1998</v>
+        <v>1997</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>48</v>
@@ -7178,7 +7175,7 @@
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>1999</v>
+        <v>1998</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>47</v>
@@ -7538,34 +7535,34 @@
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>2000</v>
+        <v>1999</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>2017</v>
+        <v>2016</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>2001</v>
+        <v>2000</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>2018</v>
+        <v>2017</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>2002</v>
+        <v>2001</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>2019</v>
+        <v>2018</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>2003</v>
+        <v>2002</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>2020</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.25">
@@ -7578,18 +7575,18 @@
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>2004</v>
+        <v>2003</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>2021</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>2005</v>
+        <v>2004</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>2022</v>
+        <v>2021</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.25">
@@ -8789,7 +8786,7 @@
         <v>590</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>2023</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="282" spans="1:2" x14ac:dyDescent="0.25">
@@ -9090,18 +9087,18 @@
     </row>
     <row r="319" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A319" s="2" t="s">
-        <v>2006</v>
+        <v>2005</v>
       </c>
       <c r="B319" s="2" t="s">
-        <v>2006</v>
+        <v>2005</v>
       </c>
     </row>
     <row r="320" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A320" s="2" t="s">
-        <v>2007</v>
+        <v>2006</v>
       </c>
       <c r="B320" s="2" t="s">
-        <v>2007</v>
+        <v>2006</v>
       </c>
     </row>
     <row r="321" spans="1:2" x14ac:dyDescent="0.25">
@@ -9306,10 +9303,10 @@
     </row>
     <row r="346" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A346" s="2" t="s">
-        <v>2008</v>
+        <v>2007</v>
       </c>
       <c r="B346" s="2" t="s">
-        <v>2008</v>
+        <v>2007</v>
       </c>
     </row>
     <row r="347" spans="1:2" x14ac:dyDescent="0.25">
@@ -9357,7 +9354,7 @@
         <v>1877</v>
       </c>
       <c r="B352" s="2" t="s">
-        <v>2024</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="353" spans="1:2" x14ac:dyDescent="0.25">
@@ -9717,7 +9714,7 @@
         <v>1720</v>
       </c>
       <c r="B397" s="2" t="s">
-        <v>2025</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="398" spans="1:2" x14ac:dyDescent="0.25">
@@ -9869,7 +9866,7 @@
         <v>1380</v>
       </c>
       <c r="B416" s="2" t="s">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="417" spans="1:2" x14ac:dyDescent="0.25">
@@ -10181,7 +10178,7 @@
         <v>947</v>
       </c>
       <c r="B455" s="2" t="s">
-        <v>2027</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="456" spans="1:2" x14ac:dyDescent="0.25">
@@ -11757,7 +11754,7 @@
         <v>1414</v>
       </c>
       <c r="B652" s="2" t="s">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="653" spans="1:2" x14ac:dyDescent="0.25">
@@ -12269,7 +12266,7 @@
         <v>1351</v>
       </c>
       <c r="B716" s="2" t="s">
-        <v>2029</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="717" spans="1:2" x14ac:dyDescent="0.25">
@@ -12314,18 +12311,18 @@
     </row>
     <row r="722" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A722" s="2" t="s">
-        <v>2009</v>
+        <v>2008</v>
       </c>
       <c r="B722" s="2" t="s">
-        <v>2030</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="723" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A723" s="2" t="s">
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="B723" s="2" t="s">
-        <v>2031</v>
+        <v>2030</v>
       </c>
     </row>
     <row r="724" spans="1:2" x14ac:dyDescent="0.25">
@@ -13501,7 +13498,7 @@
         <v>1513</v>
       </c>
       <c r="B870" s="2" t="s">
-        <v>2032</v>
+        <v>2031</v>
       </c>
     </row>
     <row r="871" spans="1:2" x14ac:dyDescent="0.25">
@@ -13594,26 +13591,26 @@
     </row>
     <row r="882" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A882" s="2" t="s">
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="B882" s="2" t="s">
-        <v>2011</v>
+        <v>2010</v>
       </c>
     </row>
     <row r="883" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A883" s="2" t="s">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="B883" s="2" t="s">
-        <v>2012</v>
+        <v>2011</v>
       </c>
     </row>
     <row r="884" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A884" s="2" t="s">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="B884" s="2" t="s">
-        <v>2013</v>
+        <v>2012</v>
       </c>
     </row>
     <row r="885" spans="1:2" x14ac:dyDescent="0.25">
@@ -14010,10 +14007,10 @@
     </row>
     <row r="934" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A934" s="2" t="s">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="B934" s="2" t="s">
-        <v>2014</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="935" spans="1:2" x14ac:dyDescent="0.25">
@@ -14674,10 +14671,10 @@
     </row>
     <row r="1017" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1017" s="2" t="s">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="B1017" s="2" t="s">
-        <v>2015</v>
+        <v>2014</v>
       </c>
     </row>
     <row r="1018" spans="1:2" x14ac:dyDescent="0.25">
@@ -14954,10 +14951,10 @@
     </row>
     <row r="1052" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1052" s="2" t="s">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="B1052" s="2" t="s">
-        <v>2033</v>
+        <v>2032</v>
       </c>
     </row>
     <row r="1053" spans="1:2" x14ac:dyDescent="0.25">
@@ -16239,7 +16236,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE2F72EB-5581-42FA-BC4C-1121F4D40726}">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
@@ -16257,17 +16254,27 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>1997</v>
+        <v>357</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>1063</v>
+        <v>531</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>1256</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>1165</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>1066</v>
       </c>
     </row>
   </sheetData>

</xml_diff>